<commit_message>
Enxuga a planilha de comissao: tira Referencia, Previsto e contrato do painel
- remove a coluna Referencia (nao serve a rotina do dia); Conferir
  passa a ser a coluna P e a aba fica com 16 colunas
- status reduzido a Em aberto e Pago: so entra na planilha o projeto
  que ja foi direcionado para ela, entao o estado Previsto nao existe
- painel sem valor de contrato: seis indicadores do ano em duas
  fileiras de tres, e a tabela mes a mes comeca no valor liquido
- com dois status, a conta do painel fecha: comissao total e
  exatamente a soma de ja paga e em aberto
- regra escrita atualizada na aba Como funciona

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K1S8HPUyosaj44kGisijyQ
</commit_message>
<xml_diff>
--- a/painel/planilhas/Valvic_Comissao_Lorrane.xlsx
+++ b/painel/planilhas/Valvic_Comissao_Lorrane.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Como funciona" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comissões'!$A$3:$Q$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comissões'!$A$3:$P$123</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Comissões'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -269,7 +269,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <font>
         <b val="1"/>
@@ -291,12 +291,6 @@
           <fgColor rgb="00FAEFDC"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color rgb="002F5D8C"/>
-      </font>
     </dxf>
     <dxf>
       <fill>
@@ -668,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q123"/>
+  <dimension ref="A1:P123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -686,8 +680,7 @@
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -780,12 +773,7 @@
           <t>Pagamento em</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Referência</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Conferir</t>
         </is>
@@ -819,8 +807,7 @@
       </c>
       <c r="N4" s="6" t="n"/>
       <c r="O4" s="11" t="n"/>
-      <c r="P4" s="6" t="n"/>
-      <c r="Q4" s="12">
+      <c r="P4" s="12">
         <f>IF($D4="","",IF($J4&gt;$D4,"custos maiores que o contrato",IF(AND($N4="Pago",$O4=""),"marcado como pago, sem a data",IF($A4="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -853,8 +840,7 @@
       </c>
       <c r="N5" s="13" t="n"/>
       <c r="O5" s="16" t="n"/>
-      <c r="P5" s="13" t="n"/>
-      <c r="Q5" s="12">
+      <c r="P5" s="12">
         <f>IF($D5="","",IF($J5&gt;$D5,"custos maiores que o contrato",IF(AND($N5="Pago",$O5=""),"marcado como pago, sem a data",IF($A5="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -887,8 +873,7 @@
       </c>
       <c r="N6" s="6" t="n"/>
       <c r="O6" s="11" t="n"/>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="12">
+      <c r="P6" s="12">
         <f>IF($D6="","",IF($J6&gt;$D6,"custos maiores que o contrato",IF(AND($N6="Pago",$O6=""),"marcado como pago, sem a data",IF($A6="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -921,8 +906,7 @@
       </c>
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="16" t="n"/>
-      <c r="P7" s="13" t="n"/>
-      <c r="Q7" s="12">
+      <c r="P7" s="12">
         <f>IF($D7="","",IF($J7&gt;$D7,"custos maiores que o contrato",IF(AND($N7="Pago",$O7=""),"marcado como pago, sem a data",IF($A7="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -955,8 +939,7 @@
       </c>
       <c r="N8" s="6" t="n"/>
       <c r="O8" s="11" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="12">
+      <c r="P8" s="12">
         <f>IF($D8="","",IF($J8&gt;$D8,"custos maiores que o contrato",IF(AND($N8="Pago",$O8=""),"marcado como pago, sem a data",IF($A8="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -989,8 +972,7 @@
       </c>
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="16" t="n"/>
-      <c r="P9" s="13" t="n"/>
-      <c r="Q9" s="12">
+      <c r="P9" s="12">
         <f>IF($D9="","",IF($J9&gt;$D9,"custos maiores que o contrato",IF(AND($N9="Pago",$O9=""),"marcado como pago, sem a data",IF($A9="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1023,8 +1005,7 @@
       </c>
       <c r="N10" s="6" t="n"/>
       <c r="O10" s="11" t="n"/>
-      <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="12">
+      <c r="P10" s="12">
         <f>IF($D10="","",IF($J10&gt;$D10,"custos maiores que o contrato",IF(AND($N10="Pago",$O10=""),"marcado como pago, sem a data",IF($A10="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1057,8 +1038,7 @@
       </c>
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="16" t="n"/>
-      <c r="P11" s="13" t="n"/>
-      <c r="Q11" s="12">
+      <c r="P11" s="12">
         <f>IF($D11="","",IF($J11&gt;$D11,"custos maiores que o contrato",IF(AND($N11="Pago",$O11=""),"marcado como pago, sem a data",IF($A11="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1091,8 +1071,7 @@
       </c>
       <c r="N12" s="6" t="n"/>
       <c r="O12" s="11" t="n"/>
-      <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="12">
+      <c r="P12" s="12">
         <f>IF($D12="","",IF($J12&gt;$D12,"custos maiores que o contrato",IF(AND($N12="Pago",$O12=""),"marcado como pago, sem a data",IF($A12="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1125,8 +1104,7 @@
       </c>
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="16" t="n"/>
-      <c r="P13" s="13" t="n"/>
-      <c r="Q13" s="12">
+      <c r="P13" s="12">
         <f>IF($D13="","",IF($J13&gt;$D13,"custos maiores que o contrato",IF(AND($N13="Pago",$O13=""),"marcado como pago, sem a data",IF($A13="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1159,8 +1137,7 @@
       </c>
       <c r="N14" s="6" t="n"/>
       <c r="O14" s="11" t="n"/>
-      <c r="P14" s="6" t="n"/>
-      <c r="Q14" s="12">
+      <c r="P14" s="12">
         <f>IF($D14="","",IF($J14&gt;$D14,"custos maiores que o contrato",IF(AND($N14="Pago",$O14=""),"marcado como pago, sem a data",IF($A14="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1193,8 +1170,7 @@
       </c>
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="16" t="n"/>
-      <c r="P15" s="13" t="n"/>
-      <c r="Q15" s="12">
+      <c r="P15" s="12">
         <f>IF($D15="","",IF($J15&gt;$D15,"custos maiores que o contrato",IF(AND($N15="Pago",$O15=""),"marcado como pago, sem a data",IF($A15="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1227,8 +1203,7 @@
       </c>
       <c r="N16" s="6" t="n"/>
       <c r="O16" s="11" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="12">
+      <c r="P16" s="12">
         <f>IF($D16="","",IF($J16&gt;$D16,"custos maiores que o contrato",IF(AND($N16="Pago",$O16=""),"marcado como pago, sem a data",IF($A16="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1261,8 +1236,7 @@
       </c>
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="16" t="n"/>
-      <c r="P17" s="13" t="n"/>
-      <c r="Q17" s="12">
+      <c r="P17" s="12">
         <f>IF($D17="","",IF($J17&gt;$D17,"custos maiores que o contrato",IF(AND($N17="Pago",$O17=""),"marcado como pago, sem a data",IF($A17="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1295,8 +1269,7 @@
       </c>
       <c r="N18" s="6" t="n"/>
       <c r="O18" s="11" t="n"/>
-      <c r="P18" s="6" t="n"/>
-      <c r="Q18" s="12">
+      <c r="P18" s="12">
         <f>IF($D18="","",IF($J18&gt;$D18,"custos maiores que o contrato",IF(AND($N18="Pago",$O18=""),"marcado como pago, sem a data",IF($A18="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1329,8 +1302,7 @@
       </c>
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="16" t="n"/>
-      <c r="P19" s="13" t="n"/>
-      <c r="Q19" s="12">
+      <c r="P19" s="12">
         <f>IF($D19="","",IF($J19&gt;$D19,"custos maiores que o contrato",IF(AND($N19="Pago",$O19=""),"marcado como pago, sem a data",IF($A19="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1363,8 +1335,7 @@
       </c>
       <c r="N20" s="6" t="n"/>
       <c r="O20" s="11" t="n"/>
-      <c r="P20" s="6" t="n"/>
-      <c r="Q20" s="12">
+      <c r="P20" s="12">
         <f>IF($D20="","",IF($J20&gt;$D20,"custos maiores que o contrato",IF(AND($N20="Pago",$O20=""),"marcado como pago, sem a data",IF($A20="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1397,8 +1368,7 @@
       </c>
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="16" t="n"/>
-      <c r="P21" s="13" t="n"/>
-      <c r="Q21" s="12">
+      <c r="P21" s="12">
         <f>IF($D21="","",IF($J21&gt;$D21,"custos maiores que o contrato",IF(AND($N21="Pago",$O21=""),"marcado como pago, sem a data",IF($A21="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1431,8 +1401,7 @@
       </c>
       <c r="N22" s="6" t="n"/>
       <c r="O22" s="11" t="n"/>
-      <c r="P22" s="6" t="n"/>
-      <c r="Q22" s="12">
+      <c r="P22" s="12">
         <f>IF($D22="","",IF($J22&gt;$D22,"custos maiores que o contrato",IF(AND($N22="Pago",$O22=""),"marcado como pago, sem a data",IF($A22="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1465,8 +1434,7 @@
       </c>
       <c r="N23" s="13" t="n"/>
       <c r="O23" s="16" t="n"/>
-      <c r="P23" s="13" t="n"/>
-      <c r="Q23" s="12">
+      <c r="P23" s="12">
         <f>IF($D23="","",IF($J23&gt;$D23,"custos maiores que o contrato",IF(AND($N23="Pago",$O23=""),"marcado como pago, sem a data",IF($A23="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1499,8 +1467,7 @@
       </c>
       <c r="N24" s="6" t="n"/>
       <c r="O24" s="11" t="n"/>
-      <c r="P24" s="6" t="n"/>
-      <c r="Q24" s="12">
+      <c r="P24" s="12">
         <f>IF($D24="","",IF($J24&gt;$D24,"custos maiores que o contrato",IF(AND($N24="Pago",$O24=""),"marcado como pago, sem a data",IF($A24="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1533,8 +1500,7 @@
       </c>
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="16" t="n"/>
-      <c r="P25" s="13" t="n"/>
-      <c r="Q25" s="12">
+      <c r="P25" s="12">
         <f>IF($D25="","",IF($J25&gt;$D25,"custos maiores que o contrato",IF(AND($N25="Pago",$O25=""),"marcado como pago, sem a data",IF($A25="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1567,8 +1533,7 @@
       </c>
       <c r="N26" s="6" t="n"/>
       <c r="O26" s="11" t="n"/>
-      <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="12">
+      <c r="P26" s="12">
         <f>IF($D26="","",IF($J26&gt;$D26,"custos maiores que o contrato",IF(AND($N26="Pago",$O26=""),"marcado como pago, sem a data",IF($A26="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1601,8 +1566,7 @@
       </c>
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="16" t="n"/>
-      <c r="P27" s="13" t="n"/>
-      <c r="Q27" s="12">
+      <c r="P27" s="12">
         <f>IF($D27="","",IF($J27&gt;$D27,"custos maiores que o contrato",IF(AND($N27="Pago",$O27=""),"marcado como pago, sem a data",IF($A27="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1635,8 +1599,7 @@
       </c>
       <c r="N28" s="6" t="n"/>
       <c r="O28" s="11" t="n"/>
-      <c r="P28" s="6" t="n"/>
-      <c r="Q28" s="12">
+      <c r="P28" s="12">
         <f>IF($D28="","",IF($J28&gt;$D28,"custos maiores que o contrato",IF(AND($N28="Pago",$O28=""),"marcado como pago, sem a data",IF($A28="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1669,8 +1632,7 @@
       </c>
       <c r="N29" s="13" t="n"/>
       <c r="O29" s="16" t="n"/>
-      <c r="P29" s="13" t="n"/>
-      <c r="Q29" s="12">
+      <c r="P29" s="12">
         <f>IF($D29="","",IF($J29&gt;$D29,"custos maiores que o contrato",IF(AND($N29="Pago",$O29=""),"marcado como pago, sem a data",IF($A29="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1703,8 +1665,7 @@
       </c>
       <c r="N30" s="6" t="n"/>
       <c r="O30" s="11" t="n"/>
-      <c r="P30" s="6" t="n"/>
-      <c r="Q30" s="12">
+      <c r="P30" s="12">
         <f>IF($D30="","",IF($J30&gt;$D30,"custos maiores que o contrato",IF(AND($N30="Pago",$O30=""),"marcado como pago, sem a data",IF($A30="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1737,8 +1698,7 @@
       </c>
       <c r="N31" s="13" t="n"/>
       <c r="O31" s="16" t="n"/>
-      <c r="P31" s="13" t="n"/>
-      <c r="Q31" s="12">
+      <c r="P31" s="12">
         <f>IF($D31="","",IF($J31&gt;$D31,"custos maiores que o contrato",IF(AND($N31="Pago",$O31=""),"marcado como pago, sem a data",IF($A31="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1771,8 +1731,7 @@
       </c>
       <c r="N32" s="6" t="n"/>
       <c r="O32" s="11" t="n"/>
-      <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="12">
+      <c r="P32" s="12">
         <f>IF($D32="","",IF($J32&gt;$D32,"custos maiores que o contrato",IF(AND($N32="Pago",$O32=""),"marcado como pago, sem a data",IF($A32="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1805,8 +1764,7 @@
       </c>
       <c r="N33" s="13" t="n"/>
       <c r="O33" s="16" t="n"/>
-      <c r="P33" s="13" t="n"/>
-      <c r="Q33" s="12">
+      <c r="P33" s="12">
         <f>IF($D33="","",IF($J33&gt;$D33,"custos maiores que o contrato",IF(AND($N33="Pago",$O33=""),"marcado como pago, sem a data",IF($A33="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1839,8 +1797,7 @@
       </c>
       <c r="N34" s="6" t="n"/>
       <c r="O34" s="11" t="n"/>
-      <c r="P34" s="6" t="n"/>
-      <c r="Q34" s="12">
+      <c r="P34" s="12">
         <f>IF($D34="","",IF($J34&gt;$D34,"custos maiores que o contrato",IF(AND($N34="Pago",$O34=""),"marcado como pago, sem a data",IF($A34="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1873,8 +1830,7 @@
       </c>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="16" t="n"/>
-      <c r="P35" s="13" t="n"/>
-      <c r="Q35" s="12">
+      <c r="P35" s="12">
         <f>IF($D35="","",IF($J35&gt;$D35,"custos maiores que o contrato",IF(AND($N35="Pago",$O35=""),"marcado como pago, sem a data",IF($A35="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1907,8 +1863,7 @@
       </c>
       <c r="N36" s="6" t="n"/>
       <c r="O36" s="11" t="n"/>
-      <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="12">
+      <c r="P36" s="12">
         <f>IF($D36="","",IF($J36&gt;$D36,"custos maiores que o contrato",IF(AND($N36="Pago",$O36=""),"marcado como pago, sem a data",IF($A36="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1941,8 +1896,7 @@
       </c>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="16" t="n"/>
-      <c r="P37" s="13" t="n"/>
-      <c r="Q37" s="12">
+      <c r="P37" s="12">
         <f>IF($D37="","",IF($J37&gt;$D37,"custos maiores que o contrato",IF(AND($N37="Pago",$O37=""),"marcado como pago, sem a data",IF($A37="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -1975,8 +1929,7 @@
       </c>
       <c r="N38" s="6" t="n"/>
       <c r="O38" s="11" t="n"/>
-      <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="12">
+      <c r="P38" s="12">
         <f>IF($D38="","",IF($J38&gt;$D38,"custos maiores que o contrato",IF(AND($N38="Pago",$O38=""),"marcado como pago, sem a data",IF($A38="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2009,8 +1962,7 @@
       </c>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="16" t="n"/>
-      <c r="P39" s="13" t="n"/>
-      <c r="Q39" s="12">
+      <c r="P39" s="12">
         <f>IF($D39="","",IF($J39&gt;$D39,"custos maiores que o contrato",IF(AND($N39="Pago",$O39=""),"marcado como pago, sem a data",IF($A39="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2043,8 +1995,7 @@
       </c>
       <c r="N40" s="6" t="n"/>
       <c r="O40" s="11" t="n"/>
-      <c r="P40" s="6" t="n"/>
-      <c r="Q40" s="12">
+      <c r="P40" s="12">
         <f>IF($D40="","",IF($J40&gt;$D40,"custos maiores que o contrato",IF(AND($N40="Pago",$O40=""),"marcado como pago, sem a data",IF($A40="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2077,8 +2028,7 @@
       </c>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="16" t="n"/>
-      <c r="P41" s="13" t="n"/>
-      <c r="Q41" s="12">
+      <c r="P41" s="12">
         <f>IF($D41="","",IF($J41&gt;$D41,"custos maiores que o contrato",IF(AND($N41="Pago",$O41=""),"marcado como pago, sem a data",IF($A41="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2111,8 +2061,7 @@
       </c>
       <c r="N42" s="6" t="n"/>
       <c r="O42" s="11" t="n"/>
-      <c r="P42" s="6" t="n"/>
-      <c r="Q42" s="12">
+      <c r="P42" s="12">
         <f>IF($D42="","",IF($J42&gt;$D42,"custos maiores que o contrato",IF(AND($N42="Pago",$O42=""),"marcado como pago, sem a data",IF($A42="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2145,8 +2094,7 @@
       </c>
       <c r="N43" s="13" t="n"/>
       <c r="O43" s="16" t="n"/>
-      <c r="P43" s="13" t="n"/>
-      <c r="Q43" s="12">
+      <c r="P43" s="12">
         <f>IF($D43="","",IF($J43&gt;$D43,"custos maiores que o contrato",IF(AND($N43="Pago",$O43=""),"marcado como pago, sem a data",IF($A43="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2179,8 +2127,7 @@
       </c>
       <c r="N44" s="6" t="n"/>
       <c r="O44" s="11" t="n"/>
-      <c r="P44" s="6" t="n"/>
-      <c r="Q44" s="12">
+      <c r="P44" s="12">
         <f>IF($D44="","",IF($J44&gt;$D44,"custos maiores que o contrato",IF(AND($N44="Pago",$O44=""),"marcado como pago, sem a data",IF($A44="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2213,8 +2160,7 @@
       </c>
       <c r="N45" s="13" t="n"/>
       <c r="O45" s="16" t="n"/>
-      <c r="P45" s="13" t="n"/>
-      <c r="Q45" s="12">
+      <c r="P45" s="12">
         <f>IF($D45="","",IF($J45&gt;$D45,"custos maiores que o contrato",IF(AND($N45="Pago",$O45=""),"marcado como pago, sem a data",IF($A45="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2247,8 +2193,7 @@
       </c>
       <c r="N46" s="6" t="n"/>
       <c r="O46" s="11" t="n"/>
-      <c r="P46" s="6" t="n"/>
-      <c r="Q46" s="12">
+      <c r="P46" s="12">
         <f>IF($D46="","",IF($J46&gt;$D46,"custos maiores que o contrato",IF(AND($N46="Pago",$O46=""),"marcado como pago, sem a data",IF($A46="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2281,8 +2226,7 @@
       </c>
       <c r="N47" s="13" t="n"/>
       <c r="O47" s="16" t="n"/>
-      <c r="P47" s="13" t="n"/>
-      <c r="Q47" s="12">
+      <c r="P47" s="12">
         <f>IF($D47="","",IF($J47&gt;$D47,"custos maiores que o contrato",IF(AND($N47="Pago",$O47=""),"marcado como pago, sem a data",IF($A47="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2315,8 +2259,7 @@
       </c>
       <c r="N48" s="6" t="n"/>
       <c r="O48" s="11" t="n"/>
-      <c r="P48" s="6" t="n"/>
-      <c r="Q48" s="12">
+      <c r="P48" s="12">
         <f>IF($D48="","",IF($J48&gt;$D48,"custos maiores que o contrato",IF(AND($N48="Pago",$O48=""),"marcado como pago, sem a data",IF($A48="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2349,8 +2292,7 @@
       </c>
       <c r="N49" s="13" t="n"/>
       <c r="O49" s="16" t="n"/>
-      <c r="P49" s="13" t="n"/>
-      <c r="Q49" s="12">
+      <c r="P49" s="12">
         <f>IF($D49="","",IF($J49&gt;$D49,"custos maiores que o contrato",IF(AND($N49="Pago",$O49=""),"marcado como pago, sem a data",IF($A49="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2383,8 +2325,7 @@
       </c>
       <c r="N50" s="6" t="n"/>
       <c r="O50" s="11" t="n"/>
-      <c r="P50" s="6" t="n"/>
-      <c r="Q50" s="12">
+      <c r="P50" s="12">
         <f>IF($D50="","",IF($J50&gt;$D50,"custos maiores que o contrato",IF(AND($N50="Pago",$O50=""),"marcado como pago, sem a data",IF($A50="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2417,8 +2358,7 @@
       </c>
       <c r="N51" s="13" t="n"/>
       <c r="O51" s="16" t="n"/>
-      <c r="P51" s="13" t="n"/>
-      <c r="Q51" s="12">
+      <c r="P51" s="12">
         <f>IF($D51="","",IF($J51&gt;$D51,"custos maiores que o contrato",IF(AND($N51="Pago",$O51=""),"marcado como pago, sem a data",IF($A51="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2451,8 +2391,7 @@
       </c>
       <c r="N52" s="6" t="n"/>
       <c r="O52" s="11" t="n"/>
-      <c r="P52" s="6" t="n"/>
-      <c r="Q52" s="12">
+      <c r="P52" s="12">
         <f>IF($D52="","",IF($J52&gt;$D52,"custos maiores que o contrato",IF(AND($N52="Pago",$O52=""),"marcado como pago, sem a data",IF($A52="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2485,8 +2424,7 @@
       </c>
       <c r="N53" s="13" t="n"/>
       <c r="O53" s="16" t="n"/>
-      <c r="P53" s="13" t="n"/>
-      <c r="Q53" s="12">
+      <c r="P53" s="12">
         <f>IF($D53="","",IF($J53&gt;$D53,"custos maiores que o contrato",IF(AND($N53="Pago",$O53=""),"marcado como pago, sem a data",IF($A53="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2519,8 +2457,7 @@
       </c>
       <c r="N54" s="6" t="n"/>
       <c r="O54" s="11" t="n"/>
-      <c r="P54" s="6" t="n"/>
-      <c r="Q54" s="12">
+      <c r="P54" s="12">
         <f>IF($D54="","",IF($J54&gt;$D54,"custos maiores que o contrato",IF(AND($N54="Pago",$O54=""),"marcado como pago, sem a data",IF($A54="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2553,8 +2490,7 @@
       </c>
       <c r="N55" s="13" t="n"/>
       <c r="O55" s="16" t="n"/>
-      <c r="P55" s="13" t="n"/>
-      <c r="Q55" s="12">
+      <c r="P55" s="12">
         <f>IF($D55="","",IF($J55&gt;$D55,"custos maiores que o contrato",IF(AND($N55="Pago",$O55=""),"marcado como pago, sem a data",IF($A55="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2587,8 +2523,7 @@
       </c>
       <c r="N56" s="6" t="n"/>
       <c r="O56" s="11" t="n"/>
-      <c r="P56" s="6" t="n"/>
-      <c r="Q56" s="12">
+      <c r="P56" s="12">
         <f>IF($D56="","",IF($J56&gt;$D56,"custos maiores que o contrato",IF(AND($N56="Pago",$O56=""),"marcado como pago, sem a data",IF($A56="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2621,8 +2556,7 @@
       </c>
       <c r="N57" s="13" t="n"/>
       <c r="O57" s="16" t="n"/>
-      <c r="P57" s="13" t="n"/>
-      <c r="Q57" s="12">
+      <c r="P57" s="12">
         <f>IF($D57="","",IF($J57&gt;$D57,"custos maiores que o contrato",IF(AND($N57="Pago",$O57=""),"marcado como pago, sem a data",IF($A57="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2655,8 +2589,7 @@
       </c>
       <c r="N58" s="6" t="n"/>
       <c r="O58" s="11" t="n"/>
-      <c r="P58" s="6" t="n"/>
-      <c r="Q58" s="12">
+      <c r="P58" s="12">
         <f>IF($D58="","",IF($J58&gt;$D58,"custos maiores que o contrato",IF(AND($N58="Pago",$O58=""),"marcado como pago, sem a data",IF($A58="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2689,8 +2622,7 @@
       </c>
       <c r="N59" s="13" t="n"/>
       <c r="O59" s="16" t="n"/>
-      <c r="P59" s="13" t="n"/>
-      <c r="Q59" s="12">
+      <c r="P59" s="12">
         <f>IF($D59="","",IF($J59&gt;$D59,"custos maiores que o contrato",IF(AND($N59="Pago",$O59=""),"marcado como pago, sem a data",IF($A59="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2723,8 +2655,7 @@
       </c>
       <c r="N60" s="6" t="n"/>
       <c r="O60" s="11" t="n"/>
-      <c r="P60" s="6" t="n"/>
-      <c r="Q60" s="12">
+      <c r="P60" s="12">
         <f>IF($D60="","",IF($J60&gt;$D60,"custos maiores que o contrato",IF(AND($N60="Pago",$O60=""),"marcado como pago, sem a data",IF($A60="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2757,8 +2688,7 @@
       </c>
       <c r="N61" s="13" t="n"/>
       <c r="O61" s="16" t="n"/>
-      <c r="P61" s="13" t="n"/>
-      <c r="Q61" s="12">
+      <c r="P61" s="12">
         <f>IF($D61="","",IF($J61&gt;$D61,"custos maiores que o contrato",IF(AND($N61="Pago",$O61=""),"marcado como pago, sem a data",IF($A61="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2791,8 +2721,7 @@
       </c>
       <c r="N62" s="6" t="n"/>
       <c r="O62" s="11" t="n"/>
-      <c r="P62" s="6" t="n"/>
-      <c r="Q62" s="12">
+      <c r="P62" s="12">
         <f>IF($D62="","",IF($J62&gt;$D62,"custos maiores que o contrato",IF(AND($N62="Pago",$O62=""),"marcado como pago, sem a data",IF($A62="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2825,8 +2754,7 @@
       </c>
       <c r="N63" s="13" t="n"/>
       <c r="O63" s="16" t="n"/>
-      <c r="P63" s="13" t="n"/>
-      <c r="Q63" s="12">
+      <c r="P63" s="12">
         <f>IF($D63="","",IF($J63&gt;$D63,"custos maiores que o contrato",IF(AND($N63="Pago",$O63=""),"marcado como pago, sem a data",IF($A63="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2859,8 +2787,7 @@
       </c>
       <c r="N64" s="6" t="n"/>
       <c r="O64" s="11" t="n"/>
-      <c r="P64" s="6" t="n"/>
-      <c r="Q64" s="12">
+      <c r="P64" s="12">
         <f>IF($D64="","",IF($J64&gt;$D64,"custos maiores que o contrato",IF(AND($N64="Pago",$O64=""),"marcado como pago, sem a data",IF($A64="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2893,8 +2820,7 @@
       </c>
       <c r="N65" s="13" t="n"/>
       <c r="O65" s="16" t="n"/>
-      <c r="P65" s="13" t="n"/>
-      <c r="Q65" s="12">
+      <c r="P65" s="12">
         <f>IF($D65="","",IF($J65&gt;$D65,"custos maiores que o contrato",IF(AND($N65="Pago",$O65=""),"marcado como pago, sem a data",IF($A65="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2927,8 +2853,7 @@
       </c>
       <c r="N66" s="6" t="n"/>
       <c r="O66" s="11" t="n"/>
-      <c r="P66" s="6" t="n"/>
-      <c r="Q66" s="12">
+      <c r="P66" s="12">
         <f>IF($D66="","",IF($J66&gt;$D66,"custos maiores que o contrato",IF(AND($N66="Pago",$O66=""),"marcado como pago, sem a data",IF($A66="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2961,8 +2886,7 @@
       </c>
       <c r="N67" s="13" t="n"/>
       <c r="O67" s="16" t="n"/>
-      <c r="P67" s="13" t="n"/>
-      <c r="Q67" s="12">
+      <c r="P67" s="12">
         <f>IF($D67="","",IF($J67&gt;$D67,"custos maiores que o contrato",IF(AND($N67="Pago",$O67=""),"marcado como pago, sem a data",IF($A67="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -2995,8 +2919,7 @@
       </c>
       <c r="N68" s="6" t="n"/>
       <c r="O68" s="11" t="n"/>
-      <c r="P68" s="6" t="n"/>
-      <c r="Q68" s="12">
+      <c r="P68" s="12">
         <f>IF($D68="","",IF($J68&gt;$D68,"custos maiores que o contrato",IF(AND($N68="Pago",$O68=""),"marcado como pago, sem a data",IF($A68="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3029,8 +2952,7 @@
       </c>
       <c r="N69" s="13" t="n"/>
       <c r="O69" s="16" t="n"/>
-      <c r="P69" s="13" t="n"/>
-      <c r="Q69" s="12">
+      <c r="P69" s="12">
         <f>IF($D69="","",IF($J69&gt;$D69,"custos maiores que o contrato",IF(AND($N69="Pago",$O69=""),"marcado como pago, sem a data",IF($A69="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3063,8 +2985,7 @@
       </c>
       <c r="N70" s="6" t="n"/>
       <c r="O70" s="11" t="n"/>
-      <c r="P70" s="6" t="n"/>
-      <c r="Q70" s="12">
+      <c r="P70" s="12">
         <f>IF($D70="","",IF($J70&gt;$D70,"custos maiores que o contrato",IF(AND($N70="Pago",$O70=""),"marcado como pago, sem a data",IF($A70="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3097,8 +3018,7 @@
       </c>
       <c r="N71" s="13" t="n"/>
       <c r="O71" s="16" t="n"/>
-      <c r="P71" s="13" t="n"/>
-      <c r="Q71" s="12">
+      <c r="P71" s="12">
         <f>IF($D71="","",IF($J71&gt;$D71,"custos maiores que o contrato",IF(AND($N71="Pago",$O71=""),"marcado como pago, sem a data",IF($A71="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3131,8 +3051,7 @@
       </c>
       <c r="N72" s="6" t="n"/>
       <c r="O72" s="11" t="n"/>
-      <c r="P72" s="6" t="n"/>
-      <c r="Q72" s="12">
+      <c r="P72" s="12">
         <f>IF($D72="","",IF($J72&gt;$D72,"custos maiores que o contrato",IF(AND($N72="Pago",$O72=""),"marcado como pago, sem a data",IF($A72="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3165,8 +3084,7 @@
       </c>
       <c r="N73" s="13" t="n"/>
       <c r="O73" s="16" t="n"/>
-      <c r="P73" s="13" t="n"/>
-      <c r="Q73" s="12">
+      <c r="P73" s="12">
         <f>IF($D73="","",IF($J73&gt;$D73,"custos maiores que o contrato",IF(AND($N73="Pago",$O73=""),"marcado como pago, sem a data",IF($A73="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3199,8 +3117,7 @@
       </c>
       <c r="N74" s="6" t="n"/>
       <c r="O74" s="11" t="n"/>
-      <c r="P74" s="6" t="n"/>
-      <c r="Q74" s="12">
+      <c r="P74" s="12">
         <f>IF($D74="","",IF($J74&gt;$D74,"custos maiores que o contrato",IF(AND($N74="Pago",$O74=""),"marcado como pago, sem a data",IF($A74="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3233,8 +3150,7 @@
       </c>
       <c r="N75" s="13" t="n"/>
       <c r="O75" s="16" t="n"/>
-      <c r="P75" s="13" t="n"/>
-      <c r="Q75" s="12">
+      <c r="P75" s="12">
         <f>IF($D75="","",IF($J75&gt;$D75,"custos maiores que o contrato",IF(AND($N75="Pago",$O75=""),"marcado como pago, sem a data",IF($A75="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3267,8 +3183,7 @@
       </c>
       <c r="N76" s="6" t="n"/>
       <c r="O76" s="11" t="n"/>
-      <c r="P76" s="6" t="n"/>
-      <c r="Q76" s="12">
+      <c r="P76" s="12">
         <f>IF($D76="","",IF($J76&gt;$D76,"custos maiores que o contrato",IF(AND($N76="Pago",$O76=""),"marcado como pago, sem a data",IF($A76="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3301,8 +3216,7 @@
       </c>
       <c r="N77" s="13" t="n"/>
       <c r="O77" s="16" t="n"/>
-      <c r="P77" s="13" t="n"/>
-      <c r="Q77" s="12">
+      <c r="P77" s="12">
         <f>IF($D77="","",IF($J77&gt;$D77,"custos maiores que o contrato",IF(AND($N77="Pago",$O77=""),"marcado como pago, sem a data",IF($A77="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3335,8 +3249,7 @@
       </c>
       <c r="N78" s="6" t="n"/>
       <c r="O78" s="11" t="n"/>
-      <c r="P78" s="6" t="n"/>
-      <c r="Q78" s="12">
+      <c r="P78" s="12">
         <f>IF($D78="","",IF($J78&gt;$D78,"custos maiores que o contrato",IF(AND($N78="Pago",$O78=""),"marcado como pago, sem a data",IF($A78="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3369,8 +3282,7 @@
       </c>
       <c r="N79" s="13" t="n"/>
       <c r="O79" s="16" t="n"/>
-      <c r="P79" s="13" t="n"/>
-      <c r="Q79" s="12">
+      <c r="P79" s="12">
         <f>IF($D79="","",IF($J79&gt;$D79,"custos maiores que o contrato",IF(AND($N79="Pago",$O79=""),"marcado como pago, sem a data",IF($A79="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3403,8 +3315,7 @@
       </c>
       <c r="N80" s="6" t="n"/>
       <c r="O80" s="11" t="n"/>
-      <c r="P80" s="6" t="n"/>
-      <c r="Q80" s="12">
+      <c r="P80" s="12">
         <f>IF($D80="","",IF($J80&gt;$D80,"custos maiores que o contrato",IF(AND($N80="Pago",$O80=""),"marcado como pago, sem a data",IF($A80="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3437,8 +3348,7 @@
       </c>
       <c r="N81" s="13" t="n"/>
       <c r="O81" s="16" t="n"/>
-      <c r="P81" s="13" t="n"/>
-      <c r="Q81" s="12">
+      <c r="P81" s="12">
         <f>IF($D81="","",IF($J81&gt;$D81,"custos maiores que o contrato",IF(AND($N81="Pago",$O81=""),"marcado como pago, sem a data",IF($A81="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3471,8 +3381,7 @@
       </c>
       <c r="N82" s="6" t="n"/>
       <c r="O82" s="11" t="n"/>
-      <c r="P82" s="6" t="n"/>
-      <c r="Q82" s="12">
+      <c r="P82" s="12">
         <f>IF($D82="","",IF($J82&gt;$D82,"custos maiores que o contrato",IF(AND($N82="Pago",$O82=""),"marcado como pago, sem a data",IF($A82="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3505,8 +3414,7 @@
       </c>
       <c r="N83" s="13" t="n"/>
       <c r="O83" s="16" t="n"/>
-      <c r="P83" s="13" t="n"/>
-      <c r="Q83" s="12">
+      <c r="P83" s="12">
         <f>IF($D83="","",IF($J83&gt;$D83,"custos maiores que o contrato",IF(AND($N83="Pago",$O83=""),"marcado como pago, sem a data",IF($A83="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3539,8 +3447,7 @@
       </c>
       <c r="N84" s="6" t="n"/>
       <c r="O84" s="11" t="n"/>
-      <c r="P84" s="6" t="n"/>
-      <c r="Q84" s="12">
+      <c r="P84" s="12">
         <f>IF($D84="","",IF($J84&gt;$D84,"custos maiores que o contrato",IF(AND($N84="Pago",$O84=""),"marcado como pago, sem a data",IF($A84="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3573,8 +3480,7 @@
       </c>
       <c r="N85" s="13" t="n"/>
       <c r="O85" s="16" t="n"/>
-      <c r="P85" s="13" t="n"/>
-      <c r="Q85" s="12">
+      <c r="P85" s="12">
         <f>IF($D85="","",IF($J85&gt;$D85,"custos maiores que o contrato",IF(AND($N85="Pago",$O85=""),"marcado como pago, sem a data",IF($A85="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3607,8 +3513,7 @@
       </c>
       <c r="N86" s="6" t="n"/>
       <c r="O86" s="11" t="n"/>
-      <c r="P86" s="6" t="n"/>
-      <c r="Q86" s="12">
+      <c r="P86" s="12">
         <f>IF($D86="","",IF($J86&gt;$D86,"custos maiores que o contrato",IF(AND($N86="Pago",$O86=""),"marcado como pago, sem a data",IF($A86="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3641,8 +3546,7 @@
       </c>
       <c r="N87" s="13" t="n"/>
       <c r="O87" s="16" t="n"/>
-      <c r="P87" s="13" t="n"/>
-      <c r="Q87" s="12">
+      <c r="P87" s="12">
         <f>IF($D87="","",IF($J87&gt;$D87,"custos maiores que o contrato",IF(AND($N87="Pago",$O87=""),"marcado como pago, sem a data",IF($A87="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3675,8 +3579,7 @@
       </c>
       <c r="N88" s="6" t="n"/>
       <c r="O88" s="11" t="n"/>
-      <c r="P88" s="6" t="n"/>
-      <c r="Q88" s="12">
+      <c r="P88" s="12">
         <f>IF($D88="","",IF($J88&gt;$D88,"custos maiores que o contrato",IF(AND($N88="Pago",$O88=""),"marcado como pago, sem a data",IF($A88="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3709,8 +3612,7 @@
       </c>
       <c r="N89" s="13" t="n"/>
       <c r="O89" s="16" t="n"/>
-      <c r="P89" s="13" t="n"/>
-      <c r="Q89" s="12">
+      <c r="P89" s="12">
         <f>IF($D89="","",IF($J89&gt;$D89,"custos maiores que o contrato",IF(AND($N89="Pago",$O89=""),"marcado como pago, sem a data",IF($A89="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3743,8 +3645,7 @@
       </c>
       <c r="N90" s="6" t="n"/>
       <c r="O90" s="11" t="n"/>
-      <c r="P90" s="6" t="n"/>
-      <c r="Q90" s="12">
+      <c r="P90" s="12">
         <f>IF($D90="","",IF($J90&gt;$D90,"custos maiores que o contrato",IF(AND($N90="Pago",$O90=""),"marcado como pago, sem a data",IF($A90="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3777,8 +3678,7 @@
       </c>
       <c r="N91" s="13" t="n"/>
       <c r="O91" s="16" t="n"/>
-      <c r="P91" s="13" t="n"/>
-      <c r="Q91" s="12">
+      <c r="P91" s="12">
         <f>IF($D91="","",IF($J91&gt;$D91,"custos maiores que o contrato",IF(AND($N91="Pago",$O91=""),"marcado como pago, sem a data",IF($A91="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3811,8 +3711,7 @@
       </c>
       <c r="N92" s="6" t="n"/>
       <c r="O92" s="11" t="n"/>
-      <c r="P92" s="6" t="n"/>
-      <c r="Q92" s="12">
+      <c r="P92" s="12">
         <f>IF($D92="","",IF($J92&gt;$D92,"custos maiores que o contrato",IF(AND($N92="Pago",$O92=""),"marcado como pago, sem a data",IF($A92="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3845,8 +3744,7 @@
       </c>
       <c r="N93" s="13" t="n"/>
       <c r="O93" s="16" t="n"/>
-      <c r="P93" s="13" t="n"/>
-      <c r="Q93" s="12">
+      <c r="P93" s="12">
         <f>IF($D93="","",IF($J93&gt;$D93,"custos maiores que o contrato",IF(AND($N93="Pago",$O93=""),"marcado como pago, sem a data",IF($A93="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3879,8 +3777,7 @@
       </c>
       <c r="N94" s="6" t="n"/>
       <c r="O94" s="11" t="n"/>
-      <c r="P94" s="6" t="n"/>
-      <c r="Q94" s="12">
+      <c r="P94" s="12">
         <f>IF($D94="","",IF($J94&gt;$D94,"custos maiores que o contrato",IF(AND($N94="Pago",$O94=""),"marcado como pago, sem a data",IF($A94="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3913,8 +3810,7 @@
       </c>
       <c r="N95" s="13" t="n"/>
       <c r="O95" s="16" t="n"/>
-      <c r="P95" s="13" t="n"/>
-      <c r="Q95" s="12">
+      <c r="P95" s="12">
         <f>IF($D95="","",IF($J95&gt;$D95,"custos maiores que o contrato",IF(AND($N95="Pago",$O95=""),"marcado como pago, sem a data",IF($A95="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3947,8 +3843,7 @@
       </c>
       <c r="N96" s="6" t="n"/>
       <c r="O96" s="11" t="n"/>
-      <c r="P96" s="6" t="n"/>
-      <c r="Q96" s="12">
+      <c r="P96" s="12">
         <f>IF($D96="","",IF($J96&gt;$D96,"custos maiores que o contrato",IF(AND($N96="Pago",$O96=""),"marcado como pago, sem a data",IF($A96="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -3981,8 +3876,7 @@
       </c>
       <c r="N97" s="13" t="n"/>
       <c r="O97" s="16" t="n"/>
-      <c r="P97" s="13" t="n"/>
-      <c r="Q97" s="12">
+      <c r="P97" s="12">
         <f>IF($D97="","",IF($J97&gt;$D97,"custos maiores que o contrato",IF(AND($N97="Pago",$O97=""),"marcado como pago, sem a data",IF($A97="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4015,8 +3909,7 @@
       </c>
       <c r="N98" s="6" t="n"/>
       <c r="O98" s="11" t="n"/>
-      <c r="P98" s="6" t="n"/>
-      <c r="Q98" s="12">
+      <c r="P98" s="12">
         <f>IF($D98="","",IF($J98&gt;$D98,"custos maiores que o contrato",IF(AND($N98="Pago",$O98=""),"marcado como pago, sem a data",IF($A98="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4049,8 +3942,7 @@
       </c>
       <c r="N99" s="13" t="n"/>
       <c r="O99" s="16" t="n"/>
-      <c r="P99" s="13" t="n"/>
-      <c r="Q99" s="12">
+      <c r="P99" s="12">
         <f>IF($D99="","",IF($J99&gt;$D99,"custos maiores que o contrato",IF(AND($N99="Pago",$O99=""),"marcado como pago, sem a data",IF($A99="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4083,8 +3975,7 @@
       </c>
       <c r="N100" s="6" t="n"/>
       <c r="O100" s="11" t="n"/>
-      <c r="P100" s="6" t="n"/>
-      <c r="Q100" s="12">
+      <c r="P100" s="12">
         <f>IF($D100="","",IF($J100&gt;$D100,"custos maiores que o contrato",IF(AND($N100="Pago",$O100=""),"marcado como pago, sem a data",IF($A100="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4117,8 +4008,7 @@
       </c>
       <c r="N101" s="13" t="n"/>
       <c r="O101" s="16" t="n"/>
-      <c r="P101" s="13" t="n"/>
-      <c r="Q101" s="12">
+      <c r="P101" s="12">
         <f>IF($D101="","",IF($J101&gt;$D101,"custos maiores que o contrato",IF(AND($N101="Pago",$O101=""),"marcado como pago, sem a data",IF($A101="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4151,8 +4041,7 @@
       </c>
       <c r="N102" s="6" t="n"/>
       <c r="O102" s="11" t="n"/>
-      <c r="P102" s="6" t="n"/>
-      <c r="Q102" s="12">
+      <c r="P102" s="12">
         <f>IF($D102="","",IF($J102&gt;$D102,"custos maiores que o contrato",IF(AND($N102="Pago",$O102=""),"marcado como pago, sem a data",IF($A102="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4185,8 +4074,7 @@
       </c>
       <c r="N103" s="13" t="n"/>
       <c r="O103" s="16" t="n"/>
-      <c r="P103" s="13" t="n"/>
-      <c r="Q103" s="12">
+      <c r="P103" s="12">
         <f>IF($D103="","",IF($J103&gt;$D103,"custos maiores que o contrato",IF(AND($N103="Pago",$O103=""),"marcado como pago, sem a data",IF($A103="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4219,8 +4107,7 @@
       </c>
       <c r="N104" s="6" t="n"/>
       <c r="O104" s="11" t="n"/>
-      <c r="P104" s="6" t="n"/>
-      <c r="Q104" s="12">
+      <c r="P104" s="12">
         <f>IF($D104="","",IF($J104&gt;$D104,"custos maiores que o contrato",IF(AND($N104="Pago",$O104=""),"marcado como pago, sem a data",IF($A104="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4253,8 +4140,7 @@
       </c>
       <c r="N105" s="13" t="n"/>
       <c r="O105" s="16" t="n"/>
-      <c r="P105" s="13" t="n"/>
-      <c r="Q105" s="12">
+      <c r="P105" s="12">
         <f>IF($D105="","",IF($J105&gt;$D105,"custos maiores que o contrato",IF(AND($N105="Pago",$O105=""),"marcado como pago, sem a data",IF($A105="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4287,8 +4173,7 @@
       </c>
       <c r="N106" s="6" t="n"/>
       <c r="O106" s="11" t="n"/>
-      <c r="P106" s="6" t="n"/>
-      <c r="Q106" s="12">
+      <c r="P106" s="12">
         <f>IF($D106="","",IF($J106&gt;$D106,"custos maiores que o contrato",IF(AND($N106="Pago",$O106=""),"marcado como pago, sem a data",IF($A106="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4321,8 +4206,7 @@
       </c>
       <c r="N107" s="13" t="n"/>
       <c r="O107" s="16" t="n"/>
-      <c r="P107" s="13" t="n"/>
-      <c r="Q107" s="12">
+      <c r="P107" s="12">
         <f>IF($D107="","",IF($J107&gt;$D107,"custos maiores que o contrato",IF(AND($N107="Pago",$O107=""),"marcado como pago, sem a data",IF($A107="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4355,8 +4239,7 @@
       </c>
       <c r="N108" s="6" t="n"/>
       <c r="O108" s="11" t="n"/>
-      <c r="P108" s="6" t="n"/>
-      <c r="Q108" s="12">
+      <c r="P108" s="12">
         <f>IF($D108="","",IF($J108&gt;$D108,"custos maiores que o contrato",IF(AND($N108="Pago",$O108=""),"marcado como pago, sem a data",IF($A108="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4389,8 +4272,7 @@
       </c>
       <c r="N109" s="13" t="n"/>
       <c r="O109" s="16" t="n"/>
-      <c r="P109" s="13" t="n"/>
-      <c r="Q109" s="12">
+      <c r="P109" s="12">
         <f>IF($D109="","",IF($J109&gt;$D109,"custos maiores que o contrato",IF(AND($N109="Pago",$O109=""),"marcado como pago, sem a data",IF($A109="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4423,8 +4305,7 @@
       </c>
       <c r="N110" s="6" t="n"/>
       <c r="O110" s="11" t="n"/>
-      <c r="P110" s="6" t="n"/>
-      <c r="Q110" s="12">
+      <c r="P110" s="12">
         <f>IF($D110="","",IF($J110&gt;$D110,"custos maiores que o contrato",IF(AND($N110="Pago",$O110=""),"marcado como pago, sem a data",IF($A110="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4457,8 +4338,7 @@
       </c>
       <c r="N111" s="13" t="n"/>
       <c r="O111" s="16" t="n"/>
-      <c r="P111" s="13" t="n"/>
-      <c r="Q111" s="12">
+      <c r="P111" s="12">
         <f>IF($D111="","",IF($J111&gt;$D111,"custos maiores que o contrato",IF(AND($N111="Pago",$O111=""),"marcado como pago, sem a data",IF($A111="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4491,8 +4371,7 @@
       </c>
       <c r="N112" s="6" t="n"/>
       <c r="O112" s="11" t="n"/>
-      <c r="P112" s="6" t="n"/>
-      <c r="Q112" s="12">
+      <c r="P112" s="12">
         <f>IF($D112="","",IF($J112&gt;$D112,"custos maiores que o contrato",IF(AND($N112="Pago",$O112=""),"marcado como pago, sem a data",IF($A112="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4525,8 +4404,7 @@
       </c>
       <c r="N113" s="13" t="n"/>
       <c r="O113" s="16" t="n"/>
-      <c r="P113" s="13" t="n"/>
-      <c r="Q113" s="12">
+      <c r="P113" s="12">
         <f>IF($D113="","",IF($J113&gt;$D113,"custos maiores que o contrato",IF(AND($N113="Pago",$O113=""),"marcado como pago, sem a data",IF($A113="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4559,8 +4437,7 @@
       </c>
       <c r="N114" s="6" t="n"/>
       <c r="O114" s="11" t="n"/>
-      <c r="P114" s="6" t="n"/>
-      <c r="Q114" s="12">
+      <c r="P114" s="12">
         <f>IF($D114="","",IF($J114&gt;$D114,"custos maiores que o contrato",IF(AND($N114="Pago",$O114=""),"marcado como pago, sem a data",IF($A114="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4593,8 +4470,7 @@
       </c>
       <c r="N115" s="13" t="n"/>
       <c r="O115" s="16" t="n"/>
-      <c r="P115" s="13" t="n"/>
-      <c r="Q115" s="12">
+      <c r="P115" s="12">
         <f>IF($D115="","",IF($J115&gt;$D115,"custos maiores que o contrato",IF(AND($N115="Pago",$O115=""),"marcado como pago, sem a data",IF($A115="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4627,8 +4503,7 @@
       </c>
       <c r="N116" s="6" t="n"/>
       <c r="O116" s="11" t="n"/>
-      <c r="P116" s="6" t="n"/>
-      <c r="Q116" s="12">
+      <c r="P116" s="12">
         <f>IF($D116="","",IF($J116&gt;$D116,"custos maiores que o contrato",IF(AND($N116="Pago",$O116=""),"marcado como pago, sem a data",IF($A116="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4661,8 +4536,7 @@
       </c>
       <c r="N117" s="13" t="n"/>
       <c r="O117" s="16" t="n"/>
-      <c r="P117" s="13" t="n"/>
-      <c r="Q117" s="12">
+      <c r="P117" s="12">
         <f>IF($D117="","",IF($J117&gt;$D117,"custos maiores que o contrato",IF(AND($N117="Pago",$O117=""),"marcado como pago, sem a data",IF($A117="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4695,8 +4569,7 @@
       </c>
       <c r="N118" s="6" t="n"/>
       <c r="O118" s="11" t="n"/>
-      <c r="P118" s="6" t="n"/>
-      <c r="Q118" s="12">
+      <c r="P118" s="12">
         <f>IF($D118="","",IF($J118&gt;$D118,"custos maiores que o contrato",IF(AND($N118="Pago",$O118=""),"marcado como pago, sem a data",IF($A118="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4729,8 +4602,7 @@
       </c>
       <c r="N119" s="13" t="n"/>
       <c r="O119" s="16" t="n"/>
-      <c r="P119" s="13" t="n"/>
-      <c r="Q119" s="12">
+      <c r="P119" s="12">
         <f>IF($D119="","",IF($J119&gt;$D119,"custos maiores que o contrato",IF(AND($N119="Pago",$O119=""),"marcado como pago, sem a data",IF($A119="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4763,8 +4635,7 @@
       </c>
       <c r="N120" s="6" t="n"/>
       <c r="O120" s="11" t="n"/>
-      <c r="P120" s="6" t="n"/>
-      <c r="Q120" s="12">
+      <c r="P120" s="12">
         <f>IF($D120="","",IF($J120&gt;$D120,"custos maiores que o contrato",IF(AND($N120="Pago",$O120=""),"marcado como pago, sem a data",IF($A120="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4797,8 +4668,7 @@
       </c>
       <c r="N121" s="13" t="n"/>
       <c r="O121" s="16" t="n"/>
-      <c r="P121" s="13" t="n"/>
-      <c r="Q121" s="12">
+      <c r="P121" s="12">
         <f>IF($D121="","",IF($J121&gt;$D121,"custos maiores que o contrato",IF(AND($N121="Pago",$O121=""),"marcado como pago, sem a data",IF($A121="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4831,8 +4701,7 @@
       </c>
       <c r="N122" s="6" t="n"/>
       <c r="O122" s="11" t="n"/>
-      <c r="P122" s="6" t="n"/>
-      <c r="Q122" s="12">
+      <c r="P122" s="12">
         <f>IF($D122="","",IF($J122&gt;$D122,"custos maiores que o contrato",IF(AND($N122="Pago",$O122=""),"marcado como pago, sem a data",IF($A122="","falta o mês",""))))</f>
         <v/>
       </c>
@@ -4865,17 +4734,16 @@
       </c>
       <c r="N123" s="13" t="n"/>
       <c r="O123" s="16" t="n"/>
-      <c r="P123" s="13" t="n"/>
-      <c r="Q123" s="12">
+      <c r="P123" s="12">
         <f>IF($D123="","",IF($J123&gt;$D123,"custos maiores que o contrato",IF(AND($N123="Pago",$O123=""),"marcado como pago, sem a data",IF($A123="","falta o mês",""))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:Q123"/>
+  <autoFilter ref="A3:P123"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <conditionalFormatting sqref="N4:N123">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -4884,13 +4752,10 @@
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>$N4="Em aberto"</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P4:P123">
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>$N4="Previsto"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q4:Q123">
-    <cfRule type="expression" priority="4" dxfId="3">
-      <formula>$Q4&lt;&gt;""</formula>
+      <formula>$P4&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -4898,7 +4763,7 @@
       <formula1>"Jan,Fev,Mar,Abr,Mai,Jun,Jul,Ago,Set,Out,Nov,Dez"</formula1>
     </dataValidation>
     <dataValidation sqref="N4:N123" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor fora da lista" error="Escolha um valor da lista." type="list">
-      <formula1>"Previsto,Em aberto,Pago"</formula1>
+      <formula1>"Em aberto,Pago"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -4914,17 +4779,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -4956,15 +4820,10 @@
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Valor de contrato</t>
+          <t>Custos de venda</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>Custos de venda</t>
-        </is>
-      </c>
-      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>Valor líquido</t>
         </is>
@@ -4976,14 +4835,10 @@
         <v/>
       </c>
       <c r="D6" s="20">
-        <f>SUM('Comissões'!$D:$D)</f>
+        <f>SUM('Comissões'!$J:$J)</f>
         <v/>
       </c>
       <c r="F6" s="20">
-        <f>SUM('Comissões'!$J:$J)</f>
-        <v/>
-      </c>
-      <c r="H6" s="20">
         <f>SUM('Comissões'!$K:$K)</f>
         <v/>
       </c>
@@ -5002,11 +4857,6 @@
       <c r="F8" s="18" t="inlineStr">
         <is>
           <t>Em aberto</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>Prevista</t>
         </is>
       </c>
     </row>
@@ -5023,10 +4873,6 @@
         <f>SUMIF('Comissões'!$N:$N,"Em aberto",'Comissões'!$M:$M)</f>
         <v/>
       </c>
-      <c r="H9" s="20">
-        <f>SUMIF('Comissões'!$N:$N,"Previsto",'Comissões'!$M:$M)</f>
-        <v/>
-      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="B11" s="17" t="inlineStr">
@@ -5048,25 +4894,20 @@
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Contrato</t>
+          <t>Líquido</t>
         </is>
       </c>
       <c r="E12" s="23" t="inlineStr">
         <is>
-          <t>Líquido</t>
+          <t>Comissão</t>
         </is>
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>Comissão</t>
+          <t>Paga</t>
         </is>
       </c>
       <c r="G12" s="23" t="inlineStr">
-        <is>
-          <t>Paga</t>
-        </is>
-      </c>
-      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>Em aberto</t>
         </is>
@@ -5083,22 +4924,18 @@
         <v/>
       </c>
       <c r="D13" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jan",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jan",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E13" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jan",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jan",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F13" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jan",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jan",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G13" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jan",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H13" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jan",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5114,22 +4951,18 @@
         <v/>
       </c>
       <c r="D14" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Fev",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Fev",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E14" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Fev",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Fev",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F14" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Fev",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Fev",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G14" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Fev",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H14" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Fev",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5145,22 +4978,18 @@
         <v/>
       </c>
       <c r="D15" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mar",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Mar",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E15" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mar",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Mar",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F15" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mar",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mar",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G15" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mar",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H15" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mar",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5176,22 +5005,18 @@
         <v/>
       </c>
       <c r="D16" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Abr",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Abr",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E16" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Abr",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Abr",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F16" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Abr",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Abr",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G16" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Abr",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H16" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Abr",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5207,22 +5032,18 @@
         <v/>
       </c>
       <c r="D17" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mai",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Mai",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E17" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mai",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Mai",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F17" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Mai",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mai",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G17" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mai",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H17" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Mai",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5238,22 +5059,18 @@
         <v/>
       </c>
       <c r="D18" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Jun",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jun",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E18" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Jun",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jun",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F18" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Jun",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jun",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G18" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jun",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H18" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jun",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5269,22 +5086,18 @@
         <v/>
       </c>
       <c r="D19" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jul",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jul",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E19" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jul",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Jul",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F19" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Jul",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jul",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G19" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jul",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H19" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Jul",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5300,22 +5113,18 @@
         <v/>
       </c>
       <c r="D20" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Ago",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Ago",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E20" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Ago",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Ago",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F20" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Ago",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Ago",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G20" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Ago",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H20" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Ago",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5331,22 +5140,18 @@
         <v/>
       </c>
       <c r="D21" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Set",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Set",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E21" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Set",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Set",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F21" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Set",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Set",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G21" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Set",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H21" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Set",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5362,22 +5167,18 @@
         <v/>
       </c>
       <c r="D22" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Out",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Out",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E22" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Out",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Out",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F22" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Out",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Out",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G22" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Out",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H22" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Out",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5393,22 +5194,18 @@
         <v/>
       </c>
       <c r="D23" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Nov",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Nov",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E23" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Nov",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Nov",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F23" s="26">
-        <f>SUMIF('Comissões'!$A:$A,"Nov",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Nov",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G23" s="26">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Nov",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H23" s="26">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Nov",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5424,22 +5221,18 @@
         <v/>
       </c>
       <c r="D24" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Dez",'Comissões'!$D:$D)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Dez",'Comissões'!$K:$K)</f>
         <v/>
       </c>
       <c r="E24" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Dez",'Comissões'!$K:$K)</f>
+        <f>SUMIF('Comissões'!$A:$A,"Dez",'Comissões'!$M:$M)</f>
         <v/>
       </c>
       <c r="F24" s="29">
-        <f>SUMIF('Comissões'!$A:$A,"Dez",'Comissões'!$M:$M)</f>
+        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Dez",'Comissões'!$N:$N,"Pago")</f>
         <v/>
       </c>
       <c r="G24" s="29">
-        <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Dez",'Comissões'!$N:$N,"Pago")</f>
-        <v/>
-      </c>
-      <c r="H24" s="29">
         <f>SUMIFS('Comissões'!$M:$M,'Comissões'!$A:$A,"Dez",'Comissões'!$N:$N,"Em aberto")</f>
         <v/>
       </c>
@@ -5470,33 +5263,25 @@
         <f>SUM(G13:G24)</f>
         <v/>
       </c>
-      <c r="H25" s="32">
-        <f>SUM(H13:H24)</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="16">
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="F6:G6"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="B11:H11"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="F8:G8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5575,7 +5360,7 @@
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>PREVISTO — o projeto está lançado mas a comissão ainda não entrou na fila de pagamento. EM ABERTO — está na fila, a pagar. PAGO — pago, com data e referência preenchidas.</t>
+          <t>EM ABERTO — a comissão está na fila, a pagar. PAGO — pago, com a data preenchida. Só entra nesta planilha o projeto que já foi direcionado para ela.</t>
         </is>
       </c>
     </row>

</xml_diff>